<commit_message>
fix: correct December SMS reports to use monthly data instead of annual totals
Issue: Cary, Crystal Lake, and NFSS financial reports contained annual data
(Jan-Dec 2025) instead of December-only monthly data, causing distribution
recommendations to show yearly income totals.

Changes:
- Replaced Cash Flow sheets in Financial Report_Final files with correct
  December monthly data for Cary, Crystal Lake, and NFSS
- Regenerated all distribution recommendation workbooks with correct values
- Cary: Net Income changed from $118,148.72 (yearly) to $8,474.94 (monthly)
- Crystal Lake: Net Income changed from $138,955.95 (yearly) to $12,339.14 (monthly)
- NFSS: Net Income changed from yearly totals to $1,936.98 (monthly)
- Altoona remained correct (was already using monthly data)

Distribution recommendations now accurately reflect December-only income
instead of full-year totals.
</commit_message>
<xml_diff>
--- a/5. SMS Reports/.Reports/12. Dec/12.2025 SMS - Cary Distribution recommendation.xlsx
+++ b/5. SMS Reports/.Reports/12. Dec/12.2025 SMS - Cary Distribution recommendation.xlsx
@@ -461,7 +461,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>38390.85</v>
+        <v>38323.5</v>
       </c>
       <c r="B3" s="2">
         <f>"as of "&amp;TEXT(DATE(2025,12,31),"mm.dd.yyyy")</f>
@@ -492,7 +492,7 @@
     <row r="6" ht="6.75" customHeight="1"/>
     <row r="7">
       <c r="A7" s="3">
-        <f>118148.72-17813.16</f>
+        <f>8474.94-1842.24</f>
         <v/>
       </c>
       <c r="B7" s="2">

</xml_diff>